<commit_message>
AJUSTE Y ACTUALIZACION PLAN DE MEJORAMIENTO
</commit_message>
<xml_diff>
--- a/data/raw/Kawak/2025.xlsx
+++ b/data/raw/Kawak/2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5f15395a9ed9a48f/Proyectos_DS/Sistema_Indicadores_Poli/data/raw/Kawak/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="8_{B34FD21E-5942-44C7-BEC5-20DF45701E1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{93C878D7-F2B9-43EC-9DCE-E55E00D96B9B}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="8_{B34FD21E-5942-44C7-BEC5-20DF45701E1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{468C7375-D35C-4D38-9BE9-4BA6E01865C8}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CF5C8F99-ADA8-44DF-B65E-B583EA4B64F8}"/>
   </bookViews>
@@ -4162,14 +4162,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1600AA31-E3D5-4986-B5AC-C7A7BAEED592}">
-  <dimension ref="A1:AA786"/>
+  <dimension ref="A1:AB786"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="27" width="9.109375" customWidth="1"/>
     <col min="28" max="256" width="8.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -4251,8 +4251,9 @@
       <c r="AA1" s="2" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="AB1" s="2"/>
+    </row>
+    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>68</v>
       </c>
@@ -4300,7 +4301,7 @@
         <v>85.3</v>
       </c>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>69</v>
       </c>
@@ -4354,7 +4355,7 @@
         <v>90.75</v>
       </c>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>73</v>
       </c>
@@ -4402,7 +4403,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>74</v>
       </c>
@@ -4450,7 +4451,7 @@
         <v>91.49</v>
       </c>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>77</v>
       </c>
@@ -4528,7 +4529,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>84</v>
       </c>
@@ -4576,7 +4577,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>85</v>
       </c>
@@ -4624,7 +4625,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>86</v>
       </c>
@@ -4672,7 +4673,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>87</v>
       </c>
@@ -4720,7 +4721,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>88</v>
       </c>
@@ -4768,7 +4769,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>89</v>
       </c>
@@ -4816,7 +4817,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>90</v>
       </c>
@@ -4864,7 +4865,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>91</v>
       </c>
@@ -4912,7 +4913,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>92</v>
       </c>
@@ -4960,7 +4961,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>94</v>
       </c>

</xml_diff>